<commit_message>
update customer upload excel
</commit_message>
<xml_diff>
--- a/template/Customer_Template.xlsx
+++ b/template/Customer_Template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Parent</t>
   </si>
@@ -56,10 +56,31 @@
     <t>State</t>
   </si>
   <si>
+    <t>Billing Name</t>
+  </si>
+  <si>
+    <t>Billing Address</t>
+  </si>
+  <si>
+    <t>Billing Address 2</t>
+  </si>
+  <si>
+    <t>Billing Address 3</t>
+  </si>
+  <si>
+    <t>Billing Address 4</t>
+  </si>
+  <si>
+    <t>Billing State</t>
+  </si>
+  <si>
     <t>Phone</t>
   </si>
   <si>
     <t>PIC</t>
+  </si>
+  <si>
+    <t>Fax</t>
   </si>
 </sst>
 </file>
@@ -1003,7 +1024,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr defaultColWidth="8.85714285714286" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.42857142857143" customWidth="1"/>
@@ -1013,11 +1034,15 @@
     <col min="5" max="5" width="8.71428571428571" customWidth="1"/>
     <col min="6" max="8" width="9.71428571428571" customWidth="1"/>
     <col min="9" max="9" width="6.14285714285714" customWidth="1"/>
-    <col min="10" max="10" width="7.28571428571429" customWidth="1"/>
-    <col min="11" max="11" width="4.42857142857143" customWidth="1"/>
+    <col min="10" max="10" width="13.1428571428571" customWidth="1"/>
+    <col min="11" max="11" width="15.2857142857143" customWidth="1"/>
+    <col min="12" max="14" width="16.8571428571429" customWidth="1"/>
+    <col min="15" max="15" width="12.4285714285714" customWidth="1"/>
+    <col min="16" max="16" width="7.28571428571429" customWidth="1"/>
+    <col min="17" max="17" width="4.42857142857143" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1050,6 +1075,27 @@
       </c>
       <c r="K1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>